<commit_message>
Update local data state
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
-  <workbookPr/>
+  <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView windowWidth="14148" windowHeight="6480"/>
+    <workbookView windowWidth="16104" windowHeight="6564"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="49">
   <si>
     <t>名字</t>
   </si>
@@ -136,28 +136,22 @@
     <t>0503</t>
   </si>
   <si>
-    <t>郭志霖</t>
-  </si>
-  <si>
-    <t>福建省</t>
+    <t>谢蜜莲</t>
+  </si>
+  <si>
+    <t>雅加达双鱼座樱桃珊瑚</t>
+  </si>
+  <si>
+    <t>0430</t>
+  </si>
+  <si>
+    <t>周琪</t>
+  </si>
+  <si>
+    <t>QQZZ</t>
   </si>
   <si>
     <t>0505</t>
-  </si>
-  <si>
-    <t>谢蜜莲</t>
-  </si>
-  <si>
-    <t>雅加达双鱼座樱桃珊瑚</t>
-  </si>
-  <si>
-    <t>0430</t>
-  </si>
-  <si>
-    <t>周琪</t>
-  </si>
-  <si>
-    <t>QQZZ</t>
   </si>
   <si>
     <t>x</t>
@@ -194,7 +188,14 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="20">
+  <fonts count="21">
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -649,164 +650,154 @@
     </border>
   </borders>
   <cellStyleXfs count="49">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="4">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="5">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="4">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="6">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="7">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="12" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="13" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="15" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="16" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="17" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="18" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="19" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="20" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="21" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="23" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="24" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="25" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="26" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="27" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="28" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="29" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="30" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="31" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="32" borderId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" quotePrefix="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+  <cellXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -859,7 +850,7 @@
     <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
     <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -869,9 +860,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="WPS">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="WPS">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -879,39 +870,39 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="44546A"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E7E6E6"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4874CB"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="EE822F"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="F2BA02"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="75BD42"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="30C0B4"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="E54C5E"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0026E5"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="7E1FAD"/>
+        <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="WPS">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -981,544 +972,581 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="WPS">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill>
+        <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:lumOff val="17500"/>
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
-              <a:schemeClr val="phClr"/>
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="2700000" scaled="0"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
-        <a:gradFill>
+        <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:hueOff val="-2520000"/>
+                <a:tint val="100000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
-              <a:schemeClr val="phClr"/>
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="2700000" scaled="0"/>
+          <a:lin ang="16200000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
-          <a:gradFill>
-            <a:gsLst>
-              <a:gs pos="0">
-                <a:schemeClr val="phClr">
-                  <a:hueOff val="-4200000"/>
-                </a:schemeClr>
-              </a:gs>
-              <a:gs pos="100000">
-                <a:schemeClr val="phClr"/>
-              </a:gs>
-            </a:gsLst>
-            <a:lin ang="2700000" scaled="1"/>
-          </a:gradFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="101600" dist="50800" dir="5400000" algn="ctr" rotWithShape="0">
-              <a:schemeClr val="phClr">
-                <a:alpha val="60000"/>
-              </a:schemeClr>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:reflection stA="50000" endA="300" endPos="40000" dist="25400" dir="5400000" sy="-100000" algn="bl" rotWithShape="0"/>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
           </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
+                <a:alpha val="35000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
-          </a:schemeClr>
-        </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="40000">
               <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:spDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="3">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </a:style>
+    </a:spDef>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:J12"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
+  <dimension ref="A1:J11"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.6"/>
   <cols>
-    <col min="1" max="1" width="9" style="1"/>
-    <col min="2" max="2" width="26.2222222222222" style="1" customWidth="1"/>
-    <col min="3" max="3" width="9.55555555555556" style="1" customWidth="1"/>
-    <col min="4" max="4" width="16.6666666666667" style="1" customWidth="1"/>
-    <col min="5" max="16384" width="9" style="1"/>
+    <col min="8" max="8" width="13.6" customWidth="1"/>
+    <col min="9" max="9" width="12.1" customWidth="1"/>
+    <col min="10" max="10" width="6.9" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:10">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" t="s">
         <v>11</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" t="s">
         <v>12</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" t="s">
         <v>13</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="F2" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="1">
+      <c r="G2">
         <v>1</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="H2" t="s">
         <v>15</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="I2" t="s">
         <v>16</v>
       </c>
-      <c r="J2" s="1">
-        <v>213</v>
+      <c r="J2">
+        <v>413</v>
       </c>
     </row>
     <row r="3" spans="1:10">
-      <c r="A3" s="1" t="s">
+      <c r="A3" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3" t="s">
         <v>12</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="E3" t="s">
         <v>13</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="F3" t="s">
         <v>17</v>
       </c>
-      <c r="G3" s="1">
+      <c r="G3">
         <v>1</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="H3" t="s">
         <v>15</v>
       </c>
-      <c r="I3" s="2" t="s">
+      <c r="I3" t="s">
         <v>16</v>
       </c>
-      <c r="J3" s="1">
-        <v>200</v>
+      <c r="J3">
+        <v>430</v>
       </c>
     </row>
     <row r="4" spans="1:10">
-      <c r="A4" s="1" t="s">
+      <c r="A4" t="s">
         <v>18</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" t="s">
         <v>19</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" t="s">
         <v>20</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D4">
         <v>19822613867</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="E4" t="s">
         <v>13</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="F4" t="s">
         <v>21</v>
       </c>
-      <c r="G4" s="1">
+      <c r="G4">
         <v>4</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="H4" t="s">
         <v>22</v>
       </c>
-      <c r="I4" s="2" t="s">
+      <c r="I4" t="s">
         <v>22</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4">
         <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:10">
-      <c r="A5" s="1" t="s">
+      <c r="A5" t="s">
         <v>23</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="1">
+      <c r="D5">
         <v>17880959618</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="E5" t="s">
         <v>24</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="F5" t="s">
         <v>14</v>
       </c>
-      <c r="G5" s="1">
+      <c r="G5">
         <v>2</v>
       </c>
-      <c r="H5" s="2" t="s">
+      <c r="H5" t="s">
         <v>25</v>
       </c>
-      <c r="I5" s="2" t="s">
+      <c r="I5" t="s">
         <v>26</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5">
         <v>364</v>
       </c>
     </row>
     <row r="6" spans="1:10">
-      <c r="A6" s="1" t="s">
+      <c r="A6" t="s">
         <v>27</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="1">
+      <c r="D6">
         <v>19833158758</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="E6" t="s">
         <v>28</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="F6" t="s">
         <v>14</v>
       </c>
-      <c r="G6" s="1">
+      <c r="G6">
         <v>3</v>
       </c>
-      <c r="H6" s="2" t="s">
+      <c r="H6" t="s">
         <v>25</v>
       </c>
-      <c r="I6" s="2" t="s">
+      <c r="I6" t="s">
         <v>29</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6">
         <v>294</v>
       </c>
     </row>
     <row r="7" spans="1:10">
-      <c r="A7" s="1" t="s">
+      <c r="A7" t="s">
         <v>30</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" t="s">
         <v>31</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" t="s">
         <v>20</v>
       </c>
-      <c r="D7" s="1">
+      <c r="D7">
         <v>18982675631</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="E7" t="s">
         <v>32</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="F7" t="s">
         <v>21</v>
       </c>
-      <c r="G7" s="1">
+      <c r="G7">
         <v>2</v>
       </c>
-      <c r="H7" s="2" t="s">
+      <c r="H7" t="s">
         <v>33</v>
       </c>
-      <c r="I7" s="2" t="s">
+      <c r="I7" t="s">
         <v>34</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7">
         <v>75</v>
       </c>
     </row>
     <row r="8" spans="1:10">
-      <c r="A8" s="1" t="s">
+      <c r="A8" t="s">
         <v>35</v>
       </c>
-      <c r="B8" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D8" s="1">
-        <v>19959737819</v>
-      </c>
-      <c r="E8" s="1" t="s">
+      <c r="B8" t="s">
         <v>36</v>
       </c>
-      <c r="F8" s="1" t="s">
+      <c r="C8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D8">
+        <v>13365897912</v>
+      </c>
+      <c r="E8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F8" t="s">
         <v>21</v>
       </c>
-      <c r="G8" s="1">
+      <c r="G8">
         <v>4</v>
       </c>
-      <c r="H8" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="I8" s="2" t="s">
+      <c r="H8" t="s">
         <v>37</v>
       </c>
-      <c r="J8" s="1">
-        <v>60</v>
+      <c r="I8" t="s">
+        <v>26</v>
+      </c>
+      <c r="J8">
+        <v>110</v>
       </c>
     </row>
     <row r="9" spans="1:10">
-      <c r="A9" s="1" t="s">
+      <c r="A9" t="s">
         <v>38</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" t="s">
         <v>39</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="C9" t="s">
         <v>20</v>
       </c>
-      <c r="D9" s="1">
-        <v>13365897912</v>
-      </c>
-      <c r="E9" s="1" t="s">
+      <c r="D9">
+        <v>15912406780</v>
+      </c>
+      <c r="E9" t="s">
         <v>13</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="F9" t="s">
         <v>21</v>
       </c>
-      <c r="G9" s="1">
-        <v>4</v>
-      </c>
-      <c r="H9" s="2" t="s">
+      <c r="G9">
+        <v>3</v>
+      </c>
+      <c r="H9" t="s">
+        <v>34</v>
+      </c>
+      <c r="I9" t="s">
         <v>40</v>
       </c>
-      <c r="I9" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="J9" s="1">
-        <v>110</v>
+      <c r="J9">
+        <v>75</v>
       </c>
     </row>
     <row r="10" spans="1:10">
-      <c r="A10" s="1" t="s">
+      <c r="A10" t="s">
         <v>41</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" t="s">
         <v>42</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C10" t="s">
         <v>20</v>
       </c>
-      <c r="D10" s="1">
-        <v>15912406780</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F10" s="1" t="s">
+      <c r="D10" t="s">
+        <v>41</v>
+      </c>
+      <c r="E10" t="s">
+        <v>43</v>
+      </c>
+      <c r="F10" t="s">
         <v>21</v>
       </c>
-      <c r="G10" s="1">
-        <v>3</v>
-      </c>
-      <c r="H10" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="I10" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="J10" s="1">
-        <v>75</v>
+      <c r="G10">
+        <v>2</v>
+      </c>
+      <c r="H10" t="s">
+        <v>44</v>
+      </c>
+      <c r="I10" t="s">
+        <v>45</v>
+      </c>
+      <c r="J10">
+        <v>95</v>
       </c>
     </row>
     <row r="11" spans="1:10">
-      <c r="A11" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="C11" s="1" t="s">
+      <c r="A11" t="s">
+        <v>46</v>
+      </c>
+      <c r="B11" t="s">
+        <v>47</v>
+      </c>
+      <c r="C11" t="s">
         <v>20</v>
       </c>
-      <c r="D11" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="F11" s="1" t="s">
+      <c r="D11">
+        <v>18083896426</v>
+      </c>
+      <c r="E11" t="s">
+        <v>48</v>
+      </c>
+      <c r="F11" t="s">
         <v>21</v>
       </c>
-      <c r="G11" s="1">
-        <v>4</v>
-      </c>
-      <c r="H11" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="I11" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="J11" s="1">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10">
-      <c r="A12" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="D12" s="1">
-        <v>18083896426</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="G12" s="1">
+      <c r="G11">
         <v>1</v>
       </c>
-      <c r="H12" s="2" t="s">
+      <c r="H11" t="s">
         <v>33</v>
       </c>
-      <c r="I12" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="J12" s="1">
+      <c r="I11" t="s">
+        <v>40</v>
+      </c>
+      <c r="J11">
         <v>110</v>
       </c>
     </row>
   </sheetData>
-  <sortState ref="A2:J11">
-    <sortCondition ref="H2:H11"/>
-  </sortState>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
+  <ignoredErrors>
+    <ignoredError sqref="A1:J9 A10:F10 H10:J10 A11:J11" numberStoredAsText="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
 
@@ -1526,11 +1554,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.6"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
   <headerFooter/>
+  <ignoredErrors>
+    <ignoredError sqref="A1" numberStoredAsText="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
 
@@ -1538,10 +1568,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.6"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
   <headerFooter/>
+  <ignoredErrors>
+    <ignoredError sqref="A1" numberStoredAsText="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update to V6.85 and xlsx backup flow
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView windowWidth="16104" windowHeight="6564"/>
+    <workbookView windowWidth="18611" windowHeight="6312"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="50">
   <si>
     <t>名字</t>
   </si>
@@ -62,6 +62,9 @@
   </si>
   <si>
     <t>大馍</t>
+  </si>
+  <si>
+    <t>damo</t>
   </si>
   <si>
     <t>微信代理</t>
@@ -1184,6 +1187,8 @@
   <dimension ref="A1:J11"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.6"/>
   <cols>
+    <col min="2" max="2" width="40.7" customWidth="1"/>
+    <col min="4" max="4" width="19.8" customWidth="1"/>
     <col min="8" max="8" width="13.6" customWidth="1"/>
     <col min="9" max="9" width="12.1" customWidth="1"/>
     <col min="10" max="10" width="6.9" customWidth="1"/>
@@ -1226,31 +1231,31 @@
         <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G2">
         <v>1</v>
       </c>
       <c r="H2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="I2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J2">
-        <v>413</v>
+        <v>590</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -1258,60 +1263,60 @@
         <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G3">
         <v>1</v>
       </c>
       <c r="H3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="I3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J3">
-        <v>430</v>
+        <v>614</v>
       </c>
     </row>
     <row r="4" spans="1:10">
       <c r="A4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D4">
         <v>19822613867</v>
       </c>
       <c r="E4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G4">
         <v>4</v>
       </c>
       <c r="H4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="I4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="J4">
         <v>35</v>
@@ -1319,95 +1324,95 @@
     </row>
     <row r="5" spans="1:10">
       <c r="A5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D5">
         <v>17880959618</v>
       </c>
       <c r="E5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G5">
         <v>2</v>
       </c>
       <c r="H5" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="I5" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="J5">
-        <v>364</v>
+        <v>520</v>
       </c>
     </row>
     <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D6">
         <v>19833158758</v>
       </c>
       <c r="E6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F6" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G6">
         <v>3</v>
       </c>
       <c r="H6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="I6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="J6">
-        <v>294</v>
+        <v>420</v>
       </c>
     </row>
     <row r="7" spans="1:10">
       <c r="A7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C7" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D7">
         <v>18982675631</v>
       </c>
       <c r="E7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F7" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G7">
         <v>2</v>
       </c>
       <c r="H7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="I7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="J7">
         <v>75</v>
@@ -1415,31 +1420,31 @@
     </row>
     <row r="8" spans="1:10">
       <c r="A8" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C8" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D8">
         <v>13365897912</v>
       </c>
       <c r="E8" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G8">
         <v>4</v>
       </c>
       <c r="H8" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="I8" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="J8">
         <v>110</v>
@@ -1447,31 +1452,31 @@
     </row>
     <row r="9" spans="1:10">
       <c r="A9" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D9">
         <v>15912406780</v>
       </c>
       <c r="E9" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F9" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G9">
         <v>3</v>
       </c>
       <c r="H9" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="I9" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="J9">
         <v>75</v>
@@ -1479,31 +1484,31 @@
     </row>
     <row r="10" spans="1:10">
       <c r="A10" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B10" t="s">
+        <v>43</v>
+      </c>
+      <c r="C10" t="s">
+        <v>21</v>
+      </c>
+      <c r="D10" t="s">
         <v>42</v>
       </c>
-      <c r="C10" t="s">
-        <v>20</v>
-      </c>
-      <c r="D10" t="s">
-        <v>41</v>
-      </c>
       <c r="E10" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F10" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G10">
         <v>2</v>
       </c>
       <c r="H10" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I10" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="J10">
         <v>95</v>
@@ -1511,31 +1516,31 @@
     </row>
     <row r="11" spans="1:10">
       <c r="A11" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B11" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C11" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D11">
         <v>18083896426</v>
       </c>
       <c r="E11" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F11" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G11">
         <v>1</v>
       </c>
       <c r="H11" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="I11" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="J11">
         <v>110</v>
@@ -1545,7 +1550,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
   <ignoredErrors>
-    <ignoredError sqref="A1:J9 A10:F10 H10:J10 A11:J11" numberStoredAsText="1"/>
+    <ignoredError sqref="A7:J9 C5:I6 A5:A6 A4:J4 C2:I3 A2:A3 A1:J1 A10:F10 H10:J10 A11:J11" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>